<commit_message>
Fable 5 (low) 벤치마크 추가
150문항 전부 응답(형사법 29번 v1 파싱 실패 1건), 332.5/375점.
Excel·공개 JSON·README 표를 갱신했다. docs/ 이미지는 배포 워크플로가
재생성한다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/제15회 변호사시험 LLM 풀이.xlsx
+++ b/제15회 변호사시험 LLM 풀이.xlsx
@@ -1009,7 +1009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ44"/>
+  <dimension ref="A1:AK44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1205,6 +1205,11 @@
           <t>Gemini 3.6 Flash (low)</t>
         </is>
       </c>
+      <c r="AK2" s="85" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (low)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="70" t="n">
@@ -1315,6 +1320,9 @@
       <c r="AJ3" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AK3" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="72" t="n">
@@ -1425,6 +1433,9 @@
       <c r="AJ4" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AK4" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="72" t="n">
@@ -1535,6 +1546,9 @@
       <c r="AJ5" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AK5" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="72" t="n">
@@ -1645,6 +1659,9 @@
       <c r="AJ6" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AK6" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="72" t="n">
@@ -1753,6 +1770,9 @@
         <v>2</v>
       </c>
       <c r="AJ7" s="87" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK7" s="87" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1867,6 +1887,9 @@
       <c r="AJ8" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AK8" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="72" t="n">
@@ -1977,6 +2000,9 @@
       <c r="AJ9" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AK9" s="89" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="72" t="n">
@@ -2091,6 +2117,9 @@
       <c r="AJ10" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AK10" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="72" t="n">
@@ -2203,6 +2232,9 @@
       <c r="AJ11" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AK11" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="72" t="n">
@@ -2321,6 +2353,9 @@
       <c r="AJ12" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AK12" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="72" t="n">
@@ -2433,6 +2468,9 @@
       <c r="AJ13" s="89" t="n">
         <v>4</v>
       </c>
+      <c r="AK13" s="89" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="72" t="n">
@@ -2543,6 +2581,9 @@
       <c r="AJ14" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AK14" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="72" t="n">
@@ -2653,6 +2694,9 @@
       <c r="AJ15" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AK15" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="72" t="n">
@@ -2765,6 +2809,9 @@
       <c r="AJ16" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AK16" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="72" t="n">
@@ -2875,6 +2922,9 @@
       <c r="AJ17" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AK17" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="72" t="n">
@@ -2991,6 +3041,9 @@
       <c r="AJ18" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AK18" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="72" t="n">
@@ -3105,6 +3158,9 @@
       <c r="AJ19" s="89" t="n">
         <v>1</v>
       </c>
+      <c r="AK19" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="72" t="n">
@@ -3217,6 +3273,9 @@
       <c r="AJ20" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AK20" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="72" t="n">
@@ -3327,6 +3386,9 @@
       <c r="AJ21" s="89" t="n">
         <v>2</v>
       </c>
+      <c r="AK21" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="72" t="n">
@@ -3437,6 +3499,9 @@
       <c r="AJ22" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AK22" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="72" t="n">
@@ -3547,6 +3612,9 @@
       <c r="AJ23" s="89" t="n">
         <v>5</v>
       </c>
+      <c r="AK23" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="72" t="n">
@@ -3657,6 +3725,9 @@
       <c r="AJ24" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AK24" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="72" t="n">
@@ -3767,6 +3838,9 @@
       <c r="AJ25" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AK25" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="72" t="n">
@@ -3877,6 +3951,9 @@
       <c r="AJ26" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AK26" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="72" t="n">
@@ -3991,6 +4068,9 @@
       <c r="AJ27" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AK27" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="72" t="n">
@@ -4105,6 +4185,9 @@
       <c r="AJ28" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AK28" s="89" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="72" t="n">
@@ -4217,6 +4300,9 @@
       <c r="AJ29" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AK29" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="72" t="n">
@@ -4327,6 +4413,9 @@
       <c r="AJ30" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AK30" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="72" t="n">
@@ -4439,6 +4528,9 @@
       <c r="AJ31" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AK31" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="72" t="n">
@@ -4549,6 +4641,9 @@
       <c r="AJ32" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AK32" s="89" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="72" t="n">
@@ -4659,6 +4754,9 @@
       <c r="AJ33" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AK33" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="72" t="n">
@@ -4769,6 +4867,9 @@
       <c r="AJ34" s="89" t="n">
         <v>5</v>
       </c>
+      <c r="AK34" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="72" t="n">
@@ -4879,6 +4980,9 @@
       <c r="AJ35" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AK35" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="72" t="n">
@@ -4991,6 +5095,9 @@
       <c r="AJ36" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AK36" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="72" t="n">
@@ -5101,6 +5208,9 @@
       <c r="AJ37" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AK37" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="72" t="n">
@@ -5211,6 +5321,9 @@
       <c r="AJ38" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AK38" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="72" t="n">
@@ -5321,6 +5434,9 @@
       <c r="AJ39" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AK39" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="72" t="n">
@@ -5431,6 +5547,9 @@
       <c r="AJ40" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AK40" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="72" t="n">
@@ -5541,6 +5660,9 @@
       <c r="AJ41" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AK41" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="74" t="n">
@@ -5651,6 +5773,9 @@
       <c r="AJ42" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AK42" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="43"/>
     <row r="44">
@@ -5765,6 +5890,9 @@
       </c>
       <c r="AJ44" s="87" t="n">
         <v>87.5</v>
+      </c>
+      <c r="AK44" s="87" t="n">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -5781,7 +5909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG74"/>
+  <dimension ref="A1:AH74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5962,6 +6090,11 @@
           <t>Gemini 3.6 Flash (low)</t>
         </is>
       </c>
+      <c r="AH2" s="85" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (low)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="70" t="n">
@@ -6065,6 +6198,9 @@
       <c r="AG3" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AH3" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="72" t="n">
@@ -6168,6 +6304,9 @@
       <c r="AG4" s="89" t="n">
         <v>1</v>
       </c>
+      <c r="AH4" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="72" t="n">
@@ -6269,6 +6408,9 @@
       <c r="AG5" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AH5" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="72" t="n">
@@ -6370,6 +6512,9 @@
       <c r="AG6" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AH6" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="72" t="n">
@@ -6469,6 +6614,9 @@
         <v>1</v>
       </c>
       <c r="AG7" s="87" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH7" s="87" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6574,6 +6722,9 @@
       <c r="AG8" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AH8" s="89" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="72" t="n">
@@ -6677,6 +6828,9 @@
       <c r="AG9" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AH9" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="72" t="n">
@@ -6778,6 +6932,9 @@
       <c r="AG10" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AH10" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="72" t="n">
@@ -6885,6 +7042,9 @@
       <c r="AG11" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AH11" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="72" t="n">
@@ -6988,6 +7148,9 @@
       <c r="AG12" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AH12" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="72" t="n">
@@ -7089,6 +7252,9 @@
       <c r="AG13" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AH13" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="72" t="n">
@@ -7190,6 +7356,9 @@
       <c r="AG14" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AH14" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="72" t="n">
@@ -7291,6 +7460,9 @@
       <c r="AG15" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AH15" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="72" t="n">
@@ -7394,6 +7566,9 @@
       <c r="AG16" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AH16" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="72" t="n">
@@ -7499,6 +7674,9 @@
       <c r="AG17" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AH17" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="72" t="n">
@@ -7604,6 +7782,9 @@
       <c r="AG18" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AH18" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="72" t="n">
@@ -7705,6 +7886,9 @@
       <c r="AG19" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AH19" s="89" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="72" t="n">
@@ -7806,6 +7990,9 @@
       <c r="AG20" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AH20" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="72" t="n">
@@ -7909,6 +8096,9 @@
       <c r="AG21" s="89" t="n">
         <v>2</v>
       </c>
+      <c r="AH21" s="89" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="72" t="n">
@@ -8012,6 +8202,9 @@
       <c r="AG22" s="89" t="n">
         <v>3</v>
       </c>
+      <c r="AH22" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="72" t="n">
@@ -8113,6 +8306,9 @@
       <c r="AG23" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AH23" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="72" t="n">
@@ -8218,6 +8414,9 @@
       <c r="AG24" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AH24" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="72" t="n">
@@ -8321,6 +8520,9 @@
       <c r="AG25" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AH25" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="72" t="n">
@@ -8424,6 +8626,9 @@
       <c r="AG26" s="89" t="n">
         <v>5</v>
       </c>
+      <c r="AH26" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="72" t="n">
@@ -8531,6 +8736,9 @@
       <c r="AG27" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AH27" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="72" t="n">
@@ -8634,6 +8842,9 @@
       <c r="AG28" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AH28" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="72" t="n">
@@ -8735,6 +8946,9 @@
       <c r="AG29" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AH29" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="72" t="n">
@@ -8838,6 +9052,9 @@
       <c r="AG30" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AH30" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="72" t="n">
@@ -8945,6 +9162,9 @@
       <c r="AG31" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AH31" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="72" t="n">
@@ -9048,6 +9268,9 @@
       <c r="AG32" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AH32" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="72" t="n">
@@ -9151,6 +9374,9 @@
       <c r="AG33" s="89" t="n">
         <v>4</v>
       </c>
+      <c r="AH33" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="72" t="n">
@@ -9254,6 +9480,9 @@
       <c r="AG34" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AH34" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="72" t="n">
@@ -9357,6 +9586,9 @@
       <c r="AG35" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AH35" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="72" t="n">
@@ -9458,6 +9690,9 @@
       <c r="AG36" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AH36" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="72" t="n">
@@ -9559,6 +9794,9 @@
       <c r="AG37" s="89" t="n">
         <v>1</v>
       </c>
+      <c r="AH37" s="89" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="72" t="n">
@@ -9664,6 +9902,9 @@
       <c r="AG38" s="89" t="n">
         <v>5</v>
       </c>
+      <c r="AH38" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="72" t="n">
@@ -9767,6 +10008,9 @@
       <c r="AG39" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AH39" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="72" t="n">
@@ -9868,6 +10112,9 @@
       <c r="AG40" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AH40" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="72" t="n">
@@ -9973,6 +10220,9 @@
       <c r="AG41" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AH41" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="72" t="n">
@@ -10074,6 +10324,9 @@
       <c r="AG42" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AH42" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="72" t="n">
@@ -10175,6 +10428,9 @@
       <c r="AG43" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AH43" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="72" t="n">
@@ -10278,6 +10534,9 @@
       <c r="AG44" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AH44" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="72" t="n">
@@ -10379,6 +10638,9 @@
       <c r="AG45" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AH45" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="72" t="n">
@@ -10480,6 +10742,9 @@
       <c r="AG46" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AH46" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="72" t="n">
@@ -10583,6 +10848,9 @@
       <c r="AG47" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AH47" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="72" t="n">
@@ -10688,6 +10956,9 @@
       <c r="AG48" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AH48" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="72" t="n">
@@ -10789,6 +11060,9 @@
       <c r="AG49" s="89" t="n">
         <v>2</v>
       </c>
+      <c r="AH49" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="72" t="n">
@@ -10892,6 +11166,9 @@
       <c r="AG50" s="89" t="n">
         <v>2</v>
       </c>
+      <c r="AH50" s="89" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="72" t="n">
@@ -10997,6 +11274,9 @@
       <c r="AG51" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AH51" s="89" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="72" t="n">
@@ -11100,6 +11380,9 @@
       <c r="AG52" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AH52" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="72" t="n">
@@ -11205,6 +11488,9 @@
       <c r="AG53" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AH53" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="72" t="n">
@@ -11306,6 +11592,9 @@
       <c r="AG54" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AH54" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="72" t="n">
@@ -11407,6 +11696,9 @@
       <c r="AG55" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AH55" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="72" t="n">
@@ -11508,6 +11800,9 @@
       <c r="AG56" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AH56" s="89" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="72" t="n">
@@ -11609,6 +11904,9 @@
       <c r="AG57" s="89" t="n">
         <v>4</v>
       </c>
+      <c r="AH57" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="72" t="n">
@@ -11710,6 +12008,9 @@
       <c r="AG58" s="89" t="n">
         <v>2</v>
       </c>
+      <c r="AH58" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="72" t="n">
@@ -11813,6 +12114,9 @@
       <c r="AG59" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AH59" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="72" t="n">
@@ -11918,6 +12222,9 @@
       <c r="AG60" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AH60" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="72" t="n">
@@ -12019,6 +12326,9 @@
       <c r="AG61" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AH61" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="72" t="n">
@@ -12120,6 +12430,9 @@
       <c r="AG62" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AH62" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="72" t="n">
@@ -12221,6 +12534,9 @@
       <c r="AG63" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AH63" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="72" t="n">
@@ -12324,6 +12640,9 @@
       <c r="AG64" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AH64" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="72" t="n">
@@ -12425,6 +12744,9 @@
       <c r="AG65" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AH65" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="72" t="n">
@@ -12526,6 +12848,9 @@
       <c r="AG66" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AH66" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="72" t="n">
@@ -12629,6 +12954,9 @@
       <c r="AG67" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AH67" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="72" t="n">
@@ -12734,6 +13062,9 @@
       <c r="AG68" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AH68" s="89" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="72" t="n">
@@ -12835,6 +13166,9 @@
       <c r="AG69" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AH69" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="72" t="n">
@@ -12936,6 +13270,9 @@
       <c r="AG70" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AH70" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="72" t="n">
@@ -13037,6 +13374,9 @@
       <c r="AG71" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AH71" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="74" t="n">
@@ -13138,6 +13478,9 @@
       <c r="AG72" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AH72" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="73"/>
     <row r="74">
@@ -13243,6 +13586,9 @@
       </c>
       <c r="AG74" s="87" t="n">
         <v>147.5</v>
+      </c>
+      <c r="AH74" s="87" t="n">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -13259,7 +13605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI44"/>
+  <dimension ref="A1:AK44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13450,6 +13796,16 @@
           <t>Gemini 3.6 Flash (low)</t>
         </is>
       </c>
+      <c r="AJ2" s="85" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (low)</t>
+        </is>
+      </c>
+      <c r="AK2" s="85" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (low) (v2)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="70" t="n">
@@ -13561,6 +13917,12 @@
       <c r="AI3" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AJ3" s="87" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK3" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="72" t="n">
@@ -13668,6 +14030,12 @@
       <c r="AI4" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AJ4" s="87" t="n">
+        <v>4</v>
+      </c>
+      <c r="AK4" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="72" t="n">
@@ -13775,6 +14143,12 @@
       <c r="AI5" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AJ5" s="87" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK5" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="72" t="n">
@@ -13886,6 +14260,12 @@
       <c r="AI6" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AJ6" s="87" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK6" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="72" t="n">
@@ -13992,6 +14372,12 @@
       </c>
       <c r="AI7" s="87" t="n">
         <v>1</v>
+      </c>
+      <c r="AJ7" s="89" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK7" s="89" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -14104,6 +14490,12 @@
       <c r="AI8" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AJ8" s="87" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK8" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="72" t="n">
@@ -14213,6 +14605,12 @@
       <c r="AI9" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AJ9" s="87" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK9" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="72" t="n">
@@ -14320,6 +14718,12 @@
       <c r="AI10" s="89" t="n">
         <v>3</v>
       </c>
+      <c r="AJ10" s="87" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK10" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="72" t="n">
@@ -14429,6 +14833,12 @@
       <c r="AI11" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AJ11" s="87" t="n">
+        <v>4</v>
+      </c>
+      <c r="AK11" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="72" t="n">
@@ -14538,6 +14948,12 @@
       <c r="AI12" s="89" t="n">
         <v>3</v>
       </c>
+      <c r="AJ12" s="89" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK12" s="89" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="72" t="n">
@@ -14647,6 +15063,12 @@
       <c r="AI13" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AJ13" s="87" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK13" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="72" t="n">
@@ -14756,6 +15178,12 @@
       <c r="AI14" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AJ14" s="87" t="n">
+        <v>4</v>
+      </c>
+      <c r="AK14" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="72" t="n">
@@ -14863,6 +15291,12 @@
       <c r="AI15" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AJ15" s="87" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK15" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="72" t="n">
@@ -14970,6 +15404,12 @@
       <c r="AI16" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AJ16" s="87" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK16" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="72" t="n">
@@ -15085,6 +15525,12 @@
       <c r="AI17" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AJ17" s="87" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK17" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="72" t="n">
@@ -15194,6 +15640,12 @@
       <c r="AI18" s="89" t="n">
         <v>5</v>
       </c>
+      <c r="AJ18" s="87" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK18" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="72" t="n">
@@ -15303,6 +15755,12 @@
       <c r="AI19" s="87" t="n">
         <v>1</v>
       </c>
+      <c r="AJ19" s="87" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK19" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="72" t="n">
@@ -15410,6 +15868,12 @@
       <c r="AI20" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AJ20" s="87" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK20" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="72" t="n">
@@ -15519,6 +15983,12 @@
       <c r="AI21" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AJ21" s="87" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK21" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="72" t="n">
@@ -15628,6 +16098,12 @@
       <c r="AI22" s="89" t="n">
         <v>2</v>
       </c>
+      <c r="AJ22" s="87" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK22" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="72" t="n">
@@ -15737,6 +16213,12 @@
       <c r="AI23" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AJ23" s="87" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK23" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="72" t="n">
@@ -15844,6 +16326,12 @@
       <c r="AI24" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AJ24" s="87" t="n">
+        <v>4</v>
+      </c>
+      <c r="AK24" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="72" t="n">
@@ -15955,6 +16443,12 @@
       <c r="AI25" s="89" t="n">
         <v>2</v>
       </c>
+      <c r="AJ25" s="89" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK25" s="89" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="72" t="n">
@@ -16066,6 +16560,12 @@
       <c r="AI26" s="89" t="n">
         <v>5</v>
       </c>
+      <c r="AJ26" s="87" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK26" s="87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="72" t="n">
@@ -16173,6 +16673,12 @@
       <c r="AI27" s="89" t="n">
         <v>3</v>
       </c>
+      <c r="AJ27" s="87" t="n">
+        <v>4</v>
+      </c>
+      <c r="AK27" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="72" t="n">
@@ -16282,6 +16788,12 @@
       <c r="AI28" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AJ28" s="87" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK28" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="72" t="n">
@@ -16389,6 +16901,12 @@
       <c r="AI29" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AJ29" s="87" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK29" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="72" t="n">
@@ -16498,6 +17016,12 @@
       <c r="AI30" s="89" t="n">
         <v>1</v>
       </c>
+      <c r="AJ30" s="89" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK30" s="89" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="72" t="n">
@@ -16605,6 +17129,14 @@
       <c r="AI31" s="89" t="n">
         <v>4</v>
       </c>
+      <c r="AJ31" s="90" t="inlineStr">
+        <is>
+          <t>(파싱 실패)</t>
+        </is>
+      </c>
+      <c r="AK31" s="89" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="72" t="n">
@@ -16714,6 +17246,12 @@
       <c r="AI32" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AJ32" s="87" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK32" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="72" t="n">
@@ -16823,6 +17361,12 @@
       <c r="AI33" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AJ33" s="87" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK33" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="72" t="n">
@@ -16930,6 +17474,12 @@
       <c r="AI34" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AJ34" s="87" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK34" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="72" t="n">
@@ -17037,6 +17587,12 @@
       <c r="AI35" s="87" t="n">
         <v>2</v>
       </c>
+      <c r="AJ35" s="87" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK35" s="87" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="72" t="n">
@@ -17146,6 +17702,12 @@
       <c r="AI36" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AJ36" s="87" t="n">
+        <v>4</v>
+      </c>
+      <c r="AK36" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="72" t="n">
@@ -17257,6 +17819,12 @@
       <c r="AI37" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AJ37" s="87" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK37" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="72" t="n">
@@ -17364,6 +17932,12 @@
       <c r="AI38" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AJ38" s="87" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK38" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="72" t="n">
@@ -17473,6 +18047,12 @@
       <c r="AI39" s="87" t="n">
         <v>3</v>
       </c>
+      <c r="AJ39" s="87" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK39" s="87" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="72" t="n">
@@ -17584,6 +18164,12 @@
       <c r="AI40" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AJ40" s="87" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK40" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="72" t="n">
@@ -17695,6 +18281,12 @@
       <c r="AI41" s="87" t="n">
         <v>5</v>
       </c>
+      <c r="AJ41" s="87" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK41" s="87" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="74" t="n">
@@ -17802,6 +18394,12 @@
       <c r="AI42" s="87" t="n">
         <v>4</v>
       </c>
+      <c r="AJ42" s="87" t="n">
+        <v>4</v>
+      </c>
+      <c r="AK42" s="87" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="43"/>
     <row r="44">
@@ -17913,6 +18511,12 @@
       </c>
       <c r="AI44" s="87" t="n">
         <v>77.5</v>
+      </c>
+      <c r="AJ44" s="87" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="AK44" s="87" t="n">
+        <v>87.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>